<commit_message>
partial pred importance files finished for one model/epoch. small edits to rtt dtt cli code
</commit_message>
<xml_diff>
--- a/pyrate_features_binning/model_8_syn_new_pyrate_features.xlsx
+++ b/pyrate_features_binning/model_8_syn_new_pyrate_features.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\pt_diversity_rates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SimoesLabAdmin\Documents\pt_diversity_rates\pyrate_features_binning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7A0421C3-B867-4F03-B271-90226B8F69AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E9C0B56-A1A7-4E5E-B69F-9434F40685EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57510" yWindow="1200" windowWidth="28770" windowHeight="15450" xr2:uid="{1693B5E8-AE1E-4700-9D41-DCF49EBE96F4}"/>
+    <workbookView xWindow="57960" yWindow="2205" windowWidth="28440" windowHeight="12435" xr2:uid="{1693B5E8-AE1E-4700-9D41-DCF49EBE96F4}"/>
   </bookViews>
   <sheets>
     <sheet name="model_8_syn_new_pyrate_features" sheetId="1" r:id="rId1"/>

</xml_diff>